<commit_message>
updated SiouxFalls_net_DDMproj and created setup demand file to setup the demand profile
</commit_message>
<xml_diff>
--- a/SiouxFalls_net_DDMproj.xlsx
+++ b/SiouxFalls_net_DDMproj.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ucg8nb\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ucg8nb\Python Projects\PhD_Work\DynamicDecisionModels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C2F35FE-F8D8-4AB5-B444-D94762D78F6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DACEE9C-735D-4BEA-AC5D-4103ED4E3755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="20928" windowHeight="12432" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SiouxFalls_net" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="59">
   <si>
     <t>&lt;NUMBER</t>
   </si>
@@ -115,15 +115,6 @@
   </si>
   <si>
     <t>Y</t>
-  </si>
-  <si>
-    <t>standardized</t>
-  </si>
-  <si>
-    <t>Mean</t>
-  </si>
-  <si>
-    <t>Std</t>
   </si>
   <si>
     <t>name</t>
@@ -223,6 +214,9 @@
   </si>
   <si>
     <t>DOW</t>
+  </si>
+  <si>
+    <t>Nodes</t>
   </si>
 </sst>
 </file>
@@ -3838,76 +3832,76 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
         <v>28</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>29</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>30</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>31</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>32</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>33</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>34</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>35</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>36</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>37</v>
       </c>
-      <c r="K1" t="s">
+      <c r="N1" t="s">
         <v>38</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>39</v>
       </c>
-      <c r="M1" t="s">
+      <c r="P1" t="s">
         <v>40</v>
       </c>
-      <c r="N1" t="s">
+      <c r="Q1" t="s">
         <v>41</v>
       </c>
-      <c r="O1" t="s">
+      <c r="R1" t="s">
         <v>42</v>
       </c>
-      <c r="P1" t="s">
+      <c r="S1" t="s">
         <v>43</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="T1" t="s">
         <v>44</v>
       </c>
-      <c r="R1" t="s">
+      <c r="U1" t="s">
         <v>45</v>
       </c>
-      <c r="S1" t="s">
+      <c r="V1" t="s">
         <v>46</v>
       </c>
-      <c r="T1" t="s">
+      <c r="W1" t="s">
         <v>47</v>
       </c>
-      <c r="U1" t="s">
+      <c r="X1" t="s">
         <v>48</v>
-      </c>
-      <c r="V1" t="s">
-        <v>49</v>
-      </c>
-      <c r="W1" t="s">
-        <v>50</v>
-      </c>
-      <c r="X1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.55000000000000004">
@@ -3921,7 +3915,7 @@
         <v>2</v>
       </c>
       <c r="H2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I2">
         <v>1</v>
@@ -3962,7 +3956,7 @@
         <v>3</v>
       </c>
       <c r="H3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I3">
         <v>1</v>
@@ -4003,7 +3997,7 @@
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I4">
         <v>1</v>
@@ -4044,7 +4038,7 @@
         <v>6</v>
       </c>
       <c r="H5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I5">
         <v>1</v>
@@ -4085,7 +4079,7 @@
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I6">
         <v>1</v>
@@ -4126,7 +4120,7 @@
         <v>4</v>
       </c>
       <c r="H7" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I7">
         <v>1</v>
@@ -4167,7 +4161,7 @@
         <v>12</v>
       </c>
       <c r="H8" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I8">
         <v>1</v>
@@ -4208,7 +4202,7 @@
         <v>3</v>
       </c>
       <c r="H9" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I9">
         <v>1</v>
@@ -4249,7 +4243,7 @@
         <v>5</v>
       </c>
       <c r="H10" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I10">
         <v>1</v>
@@ -4290,7 +4284,7 @@
         <v>11</v>
       </c>
       <c r="H11" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I11">
         <v>1</v>
@@ -4331,7 +4325,7 @@
         <v>4</v>
       </c>
       <c r="H12" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I12">
         <v>1</v>
@@ -4372,7 +4366,7 @@
         <v>6</v>
       </c>
       <c r="H13" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I13">
         <v>1</v>
@@ -4413,7 +4407,7 @@
         <v>9</v>
       </c>
       <c r="H14" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I14">
         <v>1</v>
@@ -4454,7 +4448,7 @@
         <v>2</v>
       </c>
       <c r="H15" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I15">
         <v>1</v>
@@ -4495,7 +4489,7 @@
         <v>5</v>
       </c>
       <c r="H16" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I16">
         <v>1</v>
@@ -4536,7 +4530,7 @@
         <v>8</v>
       </c>
       <c r="H17" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I17">
         <v>1</v>
@@ -4577,7 +4571,7 @@
         <v>8</v>
       </c>
       <c r="H18" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I18">
         <v>1</v>
@@ -4618,7 +4612,7 @@
         <v>18</v>
       </c>
       <c r="H19" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I19">
         <v>1</v>
@@ -4659,7 +4653,7 @@
         <v>6</v>
       </c>
       <c r="H20" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I20">
         <v>1</v>
@@ -4700,7 +4694,7 @@
         <v>7</v>
       </c>
       <c r="H21" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I21">
         <v>1</v>
@@ -4741,7 +4735,7 @@
         <v>9</v>
       </c>
       <c r="H22" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I22">
         <v>1</v>
@@ -4782,7 +4776,7 @@
         <v>16</v>
       </c>
       <c r="H23" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I23">
         <v>1</v>
@@ -4823,7 +4817,7 @@
         <v>5</v>
       </c>
       <c r="H24" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I24">
         <v>1</v>
@@ -4864,7 +4858,7 @@
         <v>8</v>
       </c>
       <c r="H25" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I25">
         <v>1</v>
@@ -4905,7 +4899,7 @@
         <v>10</v>
       </c>
       <c r="H26" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I26">
         <v>1</v>
@@ -4946,7 +4940,7 @@
         <v>9</v>
       </c>
       <c r="H27" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I27">
         <v>1</v>
@@ -4987,7 +4981,7 @@
         <v>11</v>
       </c>
       <c r="H28" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I28">
         <v>1</v>
@@ -5028,7 +5022,7 @@
         <v>15</v>
       </c>
       <c r="H29" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I29">
         <v>1</v>
@@ -5069,7 +5063,7 @@
         <v>16</v>
       </c>
       <c r="H30" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I30">
         <v>1</v>
@@ -5110,7 +5104,7 @@
         <v>17</v>
       </c>
       <c r="H31" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I31">
         <v>1</v>
@@ -5151,7 +5145,7 @@
         <v>4</v>
       </c>
       <c r="H32" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I32">
         <v>1</v>
@@ -5192,7 +5186,7 @@
         <v>10</v>
       </c>
       <c r="H33" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I33">
         <v>1</v>
@@ -5233,7 +5227,7 @@
         <v>12</v>
       </c>
       <c r="H34" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I34">
         <v>1</v>
@@ -5274,7 +5268,7 @@
         <v>14</v>
       </c>
       <c r="H35" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I35">
         <v>1</v>
@@ -5315,7 +5309,7 @@
         <v>3</v>
       </c>
       <c r="H36" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I36">
         <v>1</v>
@@ -5356,7 +5350,7 @@
         <v>11</v>
       </c>
       <c r="H37" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I37">
         <v>1</v>
@@ -5397,7 +5391,7 @@
         <v>13</v>
       </c>
       <c r="H38" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I38">
         <v>1</v>
@@ -5438,7 +5432,7 @@
         <v>12</v>
       </c>
       <c r="H39" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I39">
         <v>1</v>
@@ -5479,7 +5473,7 @@
         <v>24</v>
       </c>
       <c r="H40" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I40">
         <v>1</v>
@@ -5520,7 +5514,7 @@
         <v>11</v>
       </c>
       <c r="H41" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I41">
         <v>1</v>
@@ -5561,7 +5555,7 @@
         <v>15</v>
       </c>
       <c r="H42" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I42">
         <v>1</v>
@@ -5602,7 +5596,7 @@
         <v>23</v>
       </c>
       <c r="H43" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I43">
         <v>1</v>
@@ -5643,7 +5637,7 @@
         <v>10</v>
       </c>
       <c r="H44" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I44">
         <v>1</v>
@@ -5684,7 +5678,7 @@
         <v>14</v>
       </c>
       <c r="H45" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I45">
         <v>1</v>
@@ -5725,7 +5719,7 @@
         <v>19</v>
       </c>
       <c r="H46" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I46">
         <v>1</v>
@@ -5766,7 +5760,7 @@
         <v>22</v>
       </c>
       <c r="H47" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I47">
         <v>1</v>
@@ -5807,7 +5801,7 @@
         <v>8</v>
       </c>
       <c r="H48" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I48">
         <v>1</v>
@@ -5848,7 +5842,7 @@
         <v>10</v>
       </c>
       <c r="H49" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I49">
         <v>1</v>
@@ -5889,7 +5883,7 @@
         <v>17</v>
       </c>
       <c r="H50" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I50">
         <v>1</v>
@@ -5930,7 +5924,7 @@
         <v>18</v>
       </c>
       <c r="H51" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I51">
         <v>1</v>
@@ -5971,7 +5965,7 @@
         <v>10</v>
       </c>
       <c r="H52" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I52">
         <v>1</v>
@@ -6012,7 +6006,7 @@
         <v>16</v>
       </c>
       <c r="H53" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I53">
         <v>1</v>
@@ -6053,7 +6047,7 @@
         <v>19</v>
       </c>
       <c r="H54" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I54">
         <v>1</v>
@@ -6094,7 +6088,7 @@
         <v>7</v>
       </c>
       <c r="H55" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I55">
         <v>1</v>
@@ -6135,7 +6129,7 @@
         <v>16</v>
       </c>
       <c r="H56" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I56">
         <v>1</v>
@@ -6176,7 +6170,7 @@
         <v>20</v>
       </c>
       <c r="H57" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I57">
         <v>1</v>
@@ -6217,7 +6211,7 @@
         <v>15</v>
       </c>
       <c r="H58" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I58">
         <v>1</v>
@@ -6258,7 +6252,7 @@
         <v>17</v>
       </c>
       <c r="H59" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I59">
         <v>1</v>
@@ -6299,7 +6293,7 @@
         <v>20</v>
       </c>
       <c r="H60" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I60">
         <v>1</v>
@@ -6340,7 +6334,7 @@
         <v>18</v>
       </c>
       <c r="H61" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I61">
         <v>1</v>
@@ -6381,7 +6375,7 @@
         <v>19</v>
       </c>
       <c r="H62" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I62">
         <v>1</v>
@@ -6422,7 +6416,7 @@
         <v>21</v>
       </c>
       <c r="H63" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I63">
         <v>1</v>
@@ -6463,7 +6457,7 @@
         <v>22</v>
       </c>
       <c r="H64" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I64">
         <v>1</v>
@@ -6504,7 +6498,7 @@
         <v>20</v>
       </c>
       <c r="H65" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I65">
         <v>1</v>
@@ -6545,7 +6539,7 @@
         <v>22</v>
       </c>
       <c r="H66" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I66">
         <v>1</v>
@@ -6586,7 +6580,7 @@
         <v>24</v>
       </c>
       <c r="H67" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I67">
         <v>1</v>
@@ -6627,7 +6621,7 @@
         <v>15</v>
       </c>
       <c r="H68" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I68">
         <v>1</v>
@@ -6668,7 +6662,7 @@
         <v>20</v>
       </c>
       <c r="H69" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I69">
         <v>1</v>
@@ -6709,7 +6703,7 @@
         <v>21</v>
       </c>
       <c r="H70" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I70">
         <v>1</v>
@@ -6750,7 +6744,7 @@
         <v>23</v>
       </c>
       <c r="H71" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I71">
         <v>1</v>
@@ -6791,7 +6785,7 @@
         <v>14</v>
       </c>
       <c r="H72" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I72">
         <v>1</v>
@@ -6832,7 +6826,7 @@
         <v>22</v>
       </c>
       <c r="H73" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I73">
         <v>1</v>
@@ -6873,7 +6867,7 @@
         <v>24</v>
       </c>
       <c r="H74" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I74">
         <v>1</v>
@@ -6914,7 +6908,7 @@
         <v>13</v>
       </c>
       <c r="H75" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I75">
         <v>1</v>
@@ -6955,7 +6949,7 @@
         <v>21</v>
       </c>
       <c r="H76" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I76">
         <v>1</v>
@@ -6996,7 +6990,7 @@
         <v>23</v>
       </c>
       <c r="H77" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="I77">
         <v>1</v>
@@ -7321,176 +7315,256 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A2:Y30"/>
+  <dimension ref="A1:Y25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="2" max="24" width="6.578125" customWidth="1"/>
     <col min="25" max="25" width="4.83984375" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1">
+        <v>1</v>
+      </c>
+      <c r="C1">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>3</v>
+      </c>
+      <c r="E1">
+        <v>4</v>
+      </c>
+      <c r="F1">
+        <v>5</v>
+      </c>
+      <c r="G1">
+        <v>6</v>
+      </c>
+      <c r="H1">
+        <v>7</v>
+      </c>
+      <c r="I1">
+        <v>8</v>
+      </c>
+      <c r="J1">
+        <v>9</v>
+      </c>
+      <c r="K1">
+        <v>10</v>
+      </c>
+      <c r="L1">
+        <v>11</v>
+      </c>
+      <c r="M1">
+        <v>12</v>
+      </c>
+      <c r="N1">
+        <v>13</v>
+      </c>
+      <c r="O1">
+        <v>14</v>
+      </c>
+      <c r="P1">
+        <v>15</v>
+      </c>
+      <c r="Q1">
+        <v>16</v>
+      </c>
+      <c r="R1">
+        <v>17</v>
+      </c>
+      <c r="S1">
+        <v>18</v>
+      </c>
+      <c r="T1">
+        <v>19</v>
+      </c>
+      <c r="U1">
+        <v>20</v>
+      </c>
+      <c r="V1">
+        <v>21</v>
+      </c>
+      <c r="W1">
+        <v>22</v>
+      </c>
+      <c r="X1">
+        <v>23</v>
+      </c>
+      <c r="Y1">
+        <v>24</v>
+      </c>
+    </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2">
+        <v>1</v>
+      </c>
       <c r="B2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="D2">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>500</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>200</v>
       </c>
       <c r="G2">
-        <v>6</v>
+        <v>300</v>
       </c>
       <c r="H2">
-        <v>7</v>
+        <v>500</v>
       </c>
       <c r="I2">
-        <v>8</v>
+        <v>800</v>
       </c>
       <c r="J2">
-        <v>9</v>
+        <v>500</v>
       </c>
       <c r="K2">
-        <v>10</v>
+        <v>1300</v>
       </c>
       <c r="L2">
-        <v>11</v>
+        <v>500</v>
       </c>
       <c r="M2">
-        <v>12</v>
+        <v>200</v>
       </c>
       <c r="N2">
-        <v>13</v>
+        <v>500</v>
       </c>
       <c r="O2">
-        <v>14</v>
+        <v>300</v>
       </c>
       <c r="P2">
-        <v>15</v>
+        <v>500</v>
       </c>
       <c r="Q2">
-        <v>16</v>
+        <v>500</v>
       </c>
       <c r="R2">
-        <v>17</v>
+        <v>400</v>
       </c>
       <c r="S2">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="T2">
-        <v>19</v>
+        <v>300</v>
       </c>
       <c r="U2">
-        <v>20</v>
+        <v>300</v>
       </c>
       <c r="V2">
-        <v>21</v>
+        <v>100</v>
       </c>
       <c r="W2">
-        <v>22</v>
+        <v>400</v>
       </c>
       <c r="X2">
-        <v>23</v>
+        <v>300</v>
       </c>
       <c r="Y2">
-        <v>24</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="C3">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>100</v>
       </c>
       <c r="E3">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F3">
+        <v>100</v>
+      </c>
+      <c r="G3">
+        <v>400</v>
+      </c>
+      <c r="H3">
         <v>200</v>
       </c>
-      <c r="G3">
+      <c r="I3">
+        <v>400</v>
+      </c>
+      <c r="J3">
+        <v>200</v>
+      </c>
+      <c r="K3">
+        <v>600</v>
+      </c>
+      <c r="L3">
+        <v>200</v>
+      </c>
+      <c r="M3">
+        <v>100</v>
+      </c>
+      <c r="N3">
         <v>300</v>
       </c>
-      <c r="H3">
-        <v>500</v>
-      </c>
-      <c r="I3">
-        <v>800</v>
-      </c>
-      <c r="J3">
-        <v>500</v>
-      </c>
-      <c r="K3">
-        <v>1300</v>
-      </c>
-      <c r="L3">
-        <v>500</v>
-      </c>
-      <c r="M3">
+      <c r="O3">
+        <v>100</v>
+      </c>
+      <c r="P3">
+        <v>100</v>
+      </c>
+      <c r="Q3">
+        <v>400</v>
+      </c>
+      <c r="R3">
         <v>200</v>
       </c>
-      <c r="N3">
-        <v>500</v>
-      </c>
-      <c r="O3">
-        <v>300</v>
-      </c>
-      <c r="P3">
-        <v>500</v>
-      </c>
-      <c r="Q3">
-        <v>500</v>
-      </c>
-      <c r="R3">
-        <v>400</v>
-      </c>
       <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
         <v>100</v>
       </c>
-      <c r="T3">
-        <v>300</v>
-      </c>
       <c r="U3">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
         <v>100</v>
       </c>
-      <c r="W3">
-        <v>400</v>
-      </c>
       <c r="X3">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="Y3">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>100</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D4">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E4">
         <v>200</v>
@@ -7499,28 +7573,28 @@
         <v>100</v>
       </c>
       <c r="G4">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="H4">
+        <v>100</v>
+      </c>
+      <c r="I4">
         <v>200</v>
       </c>
-      <c r="I4">
-        <v>400</v>
-      </c>
       <c r="J4">
+        <v>100</v>
+      </c>
+      <c r="K4">
+        <v>300</v>
+      </c>
+      <c r="L4">
+        <v>300</v>
+      </c>
+      <c r="M4">
         <v>200</v>
       </c>
-      <c r="K4">
-        <v>600</v>
-      </c>
-      <c r="L4">
-        <v>200</v>
-      </c>
-      <c r="M4">
+      <c r="N4">
         <v>100</v>
-      </c>
-      <c r="N4">
-        <v>300</v>
       </c>
       <c r="O4">
         <v>100</v>
@@ -7529,19 +7603,19 @@
         <v>100</v>
       </c>
       <c r="Q4">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="R4">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="S4">
         <v>0</v>
       </c>
       <c r="T4">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="U4">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="V4">
         <v>0</v>
@@ -7550,7 +7624,7 @@
         <v>100</v>
       </c>
       <c r="X4">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="Y4">
         <v>0</v>
@@ -7558,194 +7632,194 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5">
+        <v>500</v>
+      </c>
+      <c r="C5">
+        <v>200</v>
+      </c>
+      <c r="D5">
+        <v>200</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>500</v>
+      </c>
+      <c r="G5">
+        <v>400</v>
+      </c>
+      <c r="H5">
+        <v>400</v>
+      </c>
+      <c r="I5">
+        <v>700</v>
+      </c>
+      <c r="J5">
+        <v>700</v>
+      </c>
+      <c r="K5">
+        <v>1200</v>
+      </c>
+      <c r="L5">
+        <v>1400</v>
+      </c>
+      <c r="M5">
+        <v>600</v>
+      </c>
+      <c r="N5">
+        <v>600</v>
+      </c>
+      <c r="O5">
+        <v>500</v>
+      </c>
+      <c r="P5">
+        <v>500</v>
+      </c>
+      <c r="Q5">
+        <v>800</v>
+      </c>
+      <c r="R5">
+        <v>500</v>
+      </c>
+      <c r="S5">
         <v>100</v>
       </c>
-      <c r="C5">
-        <v>100</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
+      <c r="T5">
         <v>200</v>
       </c>
-      <c r="F5">
-        <v>100</v>
-      </c>
-      <c r="G5">
+      <c r="U5">
         <v>300</v>
       </c>
-      <c r="H5">
-        <v>100</v>
-      </c>
-      <c r="I5">
+      <c r="V5">
         <v>200</v>
       </c>
-      <c r="J5">
-        <v>100</v>
-      </c>
-      <c r="K5">
-        <v>300</v>
-      </c>
-      <c r="L5">
-        <v>300</v>
-      </c>
-      <c r="M5">
+      <c r="W5">
+        <v>400</v>
+      </c>
+      <c r="X5">
+        <v>500</v>
+      </c>
+      <c r="Y5">
         <v>200</v>
-      </c>
-      <c r="N5">
-        <v>100</v>
-      </c>
-      <c r="O5">
-        <v>100</v>
-      </c>
-      <c r="P5">
-        <v>100</v>
-      </c>
-      <c r="Q5">
-        <v>200</v>
-      </c>
-      <c r="R5">
-        <v>100</v>
-      </c>
-      <c r="S5">
-        <v>0</v>
-      </c>
-      <c r="T5">
-        <v>0</v>
-      </c>
-      <c r="U5">
-        <v>0</v>
-      </c>
-      <c r="V5">
-        <v>0</v>
-      </c>
-      <c r="W5">
-        <v>100</v>
-      </c>
-      <c r="X5">
-        <v>100</v>
-      </c>
-      <c r="Y5">
-        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6">
+        <v>200</v>
+      </c>
+      <c r="C6">
+        <v>100</v>
+      </c>
+      <c r="D6">
+        <v>100</v>
+      </c>
+      <c r="E6">
         <v>500</v>
       </c>
-      <c r="C6">
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
         <v>200</v>
       </c>
-      <c r="D6">
+      <c r="H6">
         <v>200</v>
       </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
+      <c r="I6">
         <v>500</v>
       </c>
-      <c r="G6">
-        <v>400</v>
-      </c>
-      <c r="H6">
-        <v>400</v>
-      </c>
-      <c r="I6">
-        <v>700</v>
-      </c>
       <c r="J6">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="K6">
-        <v>1200</v>
+        <v>1000</v>
       </c>
       <c r="L6">
-        <v>1400</v>
+        <v>500</v>
       </c>
       <c r="M6">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="N6">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="O6">
+        <v>100</v>
+      </c>
+      <c r="P6">
+        <v>200</v>
+      </c>
+      <c r="Q6">
         <v>500</v>
       </c>
-      <c r="P6">
-        <v>500</v>
-      </c>
-      <c r="Q6">
-        <v>800</v>
-      </c>
       <c r="R6">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
         <v>100</v>
       </c>
-      <c r="T6">
+      <c r="U6">
+        <v>100</v>
+      </c>
+      <c r="V6">
+        <v>100</v>
+      </c>
+      <c r="W6">
         <v>200</v>
       </c>
-      <c r="U6">
-        <v>300</v>
-      </c>
-      <c r="V6">
-        <v>200</v>
-      </c>
-      <c r="W6">
-        <v>400</v>
-      </c>
       <c r="X6">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="Y6">
-        <v>200</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7">
+        <v>300</v>
+      </c>
+      <c r="C7">
+        <v>400</v>
+      </c>
+      <c r="D7">
+        <v>300</v>
+      </c>
+      <c r="E7">
+        <v>400</v>
+      </c>
+      <c r="F7">
         <v>200</v>
       </c>
-      <c r="C7">
-        <v>100</v>
-      </c>
-      <c r="D7">
-        <v>100</v>
-      </c>
-      <c r="E7">
-        <v>500</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
       <c r="G7">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="H7">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="I7">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="J7">
+        <v>400</v>
+      </c>
+      <c r="K7">
         <v>800</v>
       </c>
-      <c r="K7">
-        <v>1000</v>
-      </c>
       <c r="L7">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="M7">
         <v>200</v>
@@ -7760,19 +7834,19 @@
         <v>200</v>
       </c>
       <c r="Q7">
+        <v>900</v>
+      </c>
+      <c r="R7">
         <v>500</v>
       </c>
-      <c r="R7">
+      <c r="S7">
+        <v>100</v>
+      </c>
+      <c r="T7">
         <v>200</v>
       </c>
-      <c r="S7">
-        <v>0</v>
-      </c>
-      <c r="T7">
-        <v>100</v>
-      </c>
       <c r="U7">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="V7">
         <v>100</v>
@@ -7784,21 +7858,21 @@
         <v>100</v>
       </c>
       <c r="Y7">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="C8">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="D8">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="E8">
         <v>400</v>
@@ -7807,58 +7881,58 @@
         <v>200</v>
       </c>
       <c r="G8">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>1000</v>
+      </c>
+      <c r="J8">
+        <v>600</v>
+      </c>
+      <c r="K8">
+        <v>1900</v>
+      </c>
+      <c r="L8">
+        <v>500</v>
+      </c>
+      <c r="M8">
+        <v>700</v>
+      </c>
+      <c r="N8">
         <v>400</v>
       </c>
-      <c r="I8">
-        <v>800</v>
-      </c>
-      <c r="J8">
+      <c r="O8">
+        <v>200</v>
+      </c>
+      <c r="P8">
+        <v>500</v>
+      </c>
+      <c r="Q8">
+        <v>1400</v>
+      </c>
+      <c r="R8">
+        <v>1000</v>
+      </c>
+      <c r="S8">
+        <v>200</v>
+      </c>
+      <c r="T8">
         <v>400</v>
       </c>
-      <c r="K8">
-        <v>800</v>
-      </c>
-      <c r="L8">
-        <v>400</v>
-      </c>
-      <c r="M8">
+      <c r="U8">
+        <v>500</v>
+      </c>
+      <c r="V8">
         <v>200</v>
       </c>
-      <c r="N8">
+      <c r="W8">
+        <v>500</v>
+      </c>
+      <c r="X8">
         <v>200</v>
-      </c>
-      <c r="O8">
-        <v>100</v>
-      </c>
-      <c r="P8">
-        <v>200</v>
-      </c>
-      <c r="Q8">
-        <v>900</v>
-      </c>
-      <c r="R8">
-        <v>500</v>
-      </c>
-      <c r="S8">
-        <v>100</v>
-      </c>
-      <c r="T8">
-        <v>200</v>
-      </c>
-      <c r="U8">
-        <v>300</v>
-      </c>
-      <c r="V8">
-        <v>100</v>
-      </c>
-      <c r="W8">
-        <v>200</v>
-      </c>
-      <c r="X8">
-        <v>100</v>
       </c>
       <c r="Y8">
         <v>100</v>
@@ -7866,117 +7940,117 @@
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9">
+        <v>800</v>
+      </c>
+      <c r="C9">
+        <v>400</v>
+      </c>
+      <c r="D9">
+        <v>200</v>
+      </c>
+      <c r="E9">
+        <v>700</v>
+      </c>
+      <c r="F9">
         <v>500</v>
       </c>
-      <c r="C9">
-        <v>200</v>
-      </c>
-      <c r="D9">
-        <v>100</v>
-      </c>
-      <c r="E9">
+      <c r="G9">
+        <v>800</v>
+      </c>
+      <c r="H9">
+        <v>1000</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>800</v>
+      </c>
+      <c r="K9">
+        <v>1600</v>
+      </c>
+      <c r="L9">
+        <v>800</v>
+      </c>
+      <c r="M9">
+        <v>600</v>
+      </c>
+      <c r="N9">
+        <v>600</v>
+      </c>
+      <c r="O9">
         <v>400</v>
       </c>
-      <c r="F9">
-        <v>200</v>
-      </c>
-      <c r="G9">
+      <c r="P9">
+        <v>600</v>
+      </c>
+      <c r="Q9">
+        <v>2200</v>
+      </c>
+      <c r="R9">
+        <v>1400</v>
+      </c>
+      <c r="S9">
+        <v>300</v>
+      </c>
+      <c r="T9">
+        <v>700</v>
+      </c>
+      <c r="U9">
+        <v>900</v>
+      </c>
+      <c r="V9">
         <v>400</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-      <c r="I9">
-        <v>1000</v>
-      </c>
-      <c r="J9">
-        <v>600</v>
-      </c>
-      <c r="K9">
-        <v>1900</v>
-      </c>
-      <c r="L9">
-        <v>500</v>
-      </c>
-      <c r="M9">
-        <v>700</v>
-      </c>
-      <c r="N9">
-        <v>400</v>
-      </c>
-      <c r="O9">
-        <v>200</v>
-      </c>
-      <c r="P9">
-        <v>500</v>
-      </c>
-      <c r="Q9">
-        <v>1400</v>
-      </c>
-      <c r="R9">
-        <v>1000</v>
-      </c>
-      <c r="S9">
-        <v>200</v>
-      </c>
-      <c r="T9">
-        <v>400</v>
-      </c>
-      <c r="U9">
-        <v>500</v>
-      </c>
-      <c r="V9">
-        <v>200</v>
       </c>
       <c r="W9">
         <v>500</v>
       </c>
       <c r="X9">
+        <v>300</v>
+      </c>
+      <c r="Y9">
         <v>200</v>
-      </c>
-      <c r="Y9">
-        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10">
-        <v>800</v>
+        <v>500</v>
       </c>
       <c r="C10">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="D10">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="E10">
         <v>700</v>
       </c>
       <c r="F10">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="G10">
+        <v>400</v>
+      </c>
+      <c r="H10">
+        <v>600</v>
+      </c>
+      <c r="I10">
         <v>800</v>
       </c>
-      <c r="H10">
-        <v>1000</v>
-      </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
       <c r="J10">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="K10">
-        <v>1600</v>
+        <v>2800</v>
       </c>
       <c r="L10">
-        <v>800</v>
+        <v>1400</v>
       </c>
       <c r="M10">
         <v>600</v>
@@ -7985,34 +8059,34 @@
         <v>600</v>
       </c>
       <c r="O10">
+        <v>600</v>
+      </c>
+      <c r="P10">
+        <v>900</v>
+      </c>
+      <c r="Q10">
+        <v>1400</v>
+      </c>
+      <c r="R10">
+        <v>900</v>
+      </c>
+      <c r="S10">
+        <v>200</v>
+      </c>
+      <c r="T10">
         <v>400</v>
       </c>
-      <c r="P10">
+      <c r="U10">
         <v>600</v>
       </c>
-      <c r="Q10">
-        <v>2200</v>
-      </c>
-      <c r="R10">
-        <v>1400</v>
-      </c>
-      <c r="S10">
+      <c r="V10">
         <v>300</v>
       </c>
-      <c r="T10">
+      <c r="W10">
         <v>700</v>
       </c>
-      <c r="U10">
-        <v>900</v>
-      </c>
-      <c r="V10">
-        <v>400</v>
-      </c>
-      <c r="W10">
+      <c r="X10">
         <v>500</v>
-      </c>
-      <c r="X10">
-        <v>300</v>
       </c>
       <c r="Y10">
         <v>200</v>
@@ -8020,247 +8094,247 @@
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11">
-        <v>500</v>
+        <v>1300</v>
       </c>
       <c r="C11">
-        <v>200</v>
+        <v>600</v>
       </c>
       <c r="D11">
-        <v>100</v>
+        <v>300</v>
       </c>
       <c r="E11">
+        <v>1200</v>
+      </c>
+      <c r="F11">
+        <v>1000</v>
+      </c>
+      <c r="G11">
+        <v>800</v>
+      </c>
+      <c r="H11">
+        <v>1900</v>
+      </c>
+      <c r="I11">
+        <v>1600</v>
+      </c>
+      <c r="J11">
+        <v>2800</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>4000</v>
+      </c>
+      <c r="M11">
+        <v>2000</v>
+      </c>
+      <c r="N11">
+        <v>1900</v>
+      </c>
+      <c r="O11">
+        <v>2100</v>
+      </c>
+      <c r="P11">
+        <v>4000</v>
+      </c>
+      <c r="Q11">
+        <v>4400</v>
+      </c>
+      <c r="R11">
+        <v>3900</v>
+      </c>
+      <c r="S11">
         <v>700</v>
       </c>
-      <c r="F11">
+      <c r="T11">
+        <v>1800</v>
+      </c>
+      <c r="U11">
+        <v>2500</v>
+      </c>
+      <c r="V11">
+        <v>1200</v>
+      </c>
+      <c r="W11">
+        <v>2600</v>
+      </c>
+      <c r="X11">
+        <v>1800</v>
+      </c>
+      <c r="Y11">
         <v>800</v>
-      </c>
-      <c r="G11">
-        <v>400</v>
-      </c>
-      <c r="H11">
-        <v>600</v>
-      </c>
-      <c r="I11">
-        <v>800</v>
-      </c>
-      <c r="J11">
-        <v>0</v>
-      </c>
-      <c r="K11">
-        <v>2800</v>
-      </c>
-      <c r="L11">
-        <v>1400</v>
-      </c>
-      <c r="M11">
-        <v>600</v>
-      </c>
-      <c r="N11">
-        <v>600</v>
-      </c>
-      <c r="O11">
-        <v>600</v>
-      </c>
-      <c r="P11">
-        <v>900</v>
-      </c>
-      <c r="Q11">
-        <v>1400</v>
-      </c>
-      <c r="R11">
-        <v>900</v>
-      </c>
-      <c r="S11">
-        <v>200</v>
-      </c>
-      <c r="T11">
-        <v>400</v>
-      </c>
-      <c r="U11">
-        <v>600</v>
-      </c>
-      <c r="V11">
-        <v>300</v>
-      </c>
-      <c r="W11">
-        <v>700</v>
-      </c>
-      <c r="X11">
-        <v>500</v>
-      </c>
-      <c r="Y11">
-        <v>200</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A12">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B12">
-        <v>1300</v>
+        <v>500</v>
       </c>
       <c r="C12">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="D12">
         <v>300</v>
       </c>
       <c r="E12">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="F12">
+        <v>500</v>
+      </c>
+      <c r="G12">
+        <v>400</v>
+      </c>
+      <c r="H12">
+        <v>500</v>
+      </c>
+      <c r="I12">
+        <v>800</v>
+      </c>
+      <c r="J12">
+        <v>1400</v>
+      </c>
+      <c r="K12">
+        <v>3900</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>1400</v>
+      </c>
+      <c r="N12">
         <v>1000</v>
       </c>
-      <c r="G12">
-        <v>800</v>
-      </c>
-      <c r="H12">
-        <v>1900</v>
-      </c>
-      <c r="I12">
+      <c r="O12">
         <v>1600</v>
       </c>
-      <c r="J12">
-        <v>2800</v>
-      </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
-        <v>4000</v>
-      </c>
-      <c r="M12">
-        <v>2000</v>
-      </c>
-      <c r="N12">
-        <v>1900</v>
-      </c>
-      <c r="O12">
-        <v>2100</v>
-      </c>
       <c r="P12">
-        <v>4000</v>
+        <v>1400</v>
       </c>
       <c r="Q12">
-        <v>4400</v>
+        <v>1400</v>
       </c>
       <c r="R12">
-        <v>3900</v>
+        <v>1000</v>
       </c>
       <c r="S12">
-        <v>700</v>
+        <v>100</v>
       </c>
       <c r="T12">
-        <v>1800</v>
+        <v>400</v>
       </c>
       <c r="U12">
-        <v>2500</v>
+        <v>600</v>
       </c>
       <c r="V12">
-        <v>1200</v>
+        <v>400</v>
       </c>
       <c r="W12">
-        <v>2600</v>
+        <v>1100</v>
       </c>
       <c r="X12">
-        <v>1800</v>
+        <v>1300</v>
       </c>
       <c r="Y12">
-        <v>800</v>
+        <v>600</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A13">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13">
+        <v>200</v>
+      </c>
+      <c r="C13">
+        <v>100</v>
+      </c>
+      <c r="D13">
+        <v>200</v>
+      </c>
+      <c r="E13">
+        <v>600</v>
+      </c>
+      <c r="F13">
+        <v>200</v>
+      </c>
+      <c r="G13">
+        <v>200</v>
+      </c>
+      <c r="H13">
+        <v>700</v>
+      </c>
+      <c r="I13">
+        <v>600</v>
+      </c>
+      <c r="J13">
+        <v>600</v>
+      </c>
+      <c r="K13">
+        <v>2000</v>
+      </c>
+      <c r="L13">
+        <v>1400</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>1300</v>
+      </c>
+      <c r="O13">
+        <v>700</v>
+      </c>
+      <c r="P13">
+        <v>700</v>
+      </c>
+      <c r="Q13">
+        <v>700</v>
+      </c>
+      <c r="R13">
+        <v>600</v>
+      </c>
+      <c r="S13">
+        <v>200</v>
+      </c>
+      <c r="T13">
+        <v>300</v>
+      </c>
+      <c r="U13">
+        <v>400</v>
+      </c>
+      <c r="V13">
+        <v>300</v>
+      </c>
+      <c r="W13">
+        <v>700</v>
+      </c>
+      <c r="X13">
+        <v>700</v>
+      </c>
+      <c r="Y13">
         <v>500</v>
-      </c>
-      <c r="C13">
-        <v>200</v>
-      </c>
-      <c r="D13">
-        <v>300</v>
-      </c>
-      <c r="E13">
-        <v>1500</v>
-      </c>
-      <c r="F13">
-        <v>500</v>
-      </c>
-      <c r="G13">
-        <v>400</v>
-      </c>
-      <c r="H13">
-        <v>500</v>
-      </c>
-      <c r="I13">
-        <v>800</v>
-      </c>
-      <c r="J13">
-        <v>1400</v>
-      </c>
-      <c r="K13">
-        <v>3900</v>
-      </c>
-      <c r="L13">
-        <v>0</v>
-      </c>
-      <c r="M13">
-        <v>1400</v>
-      </c>
-      <c r="N13">
-        <v>1000</v>
-      </c>
-      <c r="O13">
-        <v>1600</v>
-      </c>
-      <c r="P13">
-        <v>1400</v>
-      </c>
-      <c r="Q13">
-        <v>1400</v>
-      </c>
-      <c r="R13">
-        <v>1000</v>
-      </c>
-      <c r="S13">
-        <v>100</v>
-      </c>
-      <c r="T13">
-        <v>400</v>
-      </c>
-      <c r="U13">
-        <v>600</v>
-      </c>
-      <c r="V13">
-        <v>400</v>
-      </c>
-      <c r="W13">
-        <v>1100</v>
-      </c>
-      <c r="X13">
-        <v>1300</v>
-      </c>
-      <c r="Y13">
-        <v>600</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A14">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="C14">
+        <v>300</v>
+      </c>
+      <c r="D14">
         <v>100</v>
-      </c>
-      <c r="D14">
-        <v>200</v>
       </c>
       <c r="E14">
         <v>600</v>
@@ -8272,7 +8346,7 @@
         <v>200</v>
       </c>
       <c r="H14">
-        <v>700</v>
+        <v>400</v>
       </c>
       <c r="I14">
         <v>600</v>
@@ -8281,105 +8355,105 @@
         <v>600</v>
       </c>
       <c r="K14">
-        <v>2000</v>
+        <v>1900</v>
       </c>
       <c r="L14">
-        <v>1400</v>
+        <v>1000</v>
       </c>
       <c r="M14">
-        <v>0</v>
+        <v>1300</v>
       </c>
       <c r="N14">
-        <v>1300</v>
+        <v>0</v>
       </c>
       <c r="O14">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="P14">
         <v>700</v>
       </c>
       <c r="Q14">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="R14">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="S14">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="T14">
         <v>300</v>
       </c>
       <c r="U14">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="V14">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="W14">
-        <v>700</v>
+        <v>1300</v>
       </c>
       <c r="X14">
-        <v>700</v>
+        <v>800</v>
       </c>
       <c r="Y14">
-        <v>500</v>
+        <v>800</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A15">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="C15">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="D15">
         <v>100</v>
       </c>
       <c r="E15">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="F15">
+        <v>100</v>
+      </c>
+      <c r="G15">
+        <v>100</v>
+      </c>
+      <c r="H15">
         <v>200</v>
       </c>
-      <c r="G15">
-        <v>200</v>
-      </c>
-      <c r="H15">
+      <c r="I15">
         <v>400</v>
-      </c>
-      <c r="I15">
-        <v>600</v>
       </c>
       <c r="J15">
         <v>600</v>
       </c>
       <c r="K15">
-        <v>1900</v>
+        <v>2100</v>
       </c>
       <c r="L15">
-        <v>1000</v>
+        <v>1600</v>
       </c>
       <c r="M15">
+        <v>700</v>
+      </c>
+      <c r="N15">
+        <v>600</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
         <v>1300</v>
       </c>
-      <c r="N15">
-        <v>0</v>
-      </c>
-      <c r="O15">
-        <v>600</v>
-      </c>
-      <c r="P15">
+      <c r="Q15">
         <v>700</v>
       </c>
-      <c r="Q15">
-        <v>600</v>
-      </c>
       <c r="R15">
-        <v>500</v>
+        <v>700</v>
       </c>
       <c r="S15">
         <v>100</v>
@@ -8388,27 +8462,27 @@
         <v>300</v>
       </c>
       <c r="U15">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="V15">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="W15">
-        <v>1300</v>
+        <v>1200</v>
       </c>
       <c r="X15">
-        <v>800</v>
+        <v>1100</v>
       </c>
       <c r="Y15">
-        <v>800</v>
+        <v>400</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A16">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="C16">
         <v>100</v>
@@ -8420,61 +8494,61 @@
         <v>500</v>
       </c>
       <c r="F16">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="G16">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="H16">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="I16">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="J16">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="K16">
-        <v>2100</v>
+        <v>4000</v>
       </c>
       <c r="L16">
-        <v>1600</v>
+        <v>1400</v>
       </c>
       <c r="M16">
         <v>700</v>
       </c>
       <c r="N16">
-        <v>600</v>
+        <v>700</v>
       </c>
       <c r="O16">
-        <v>0</v>
+        <v>1300</v>
       </c>
       <c r="P16">
-        <v>1300</v>
+        <v>0</v>
       </c>
       <c r="Q16">
-        <v>700</v>
+        <v>1200</v>
       </c>
       <c r="R16">
-        <v>700</v>
+        <v>1500</v>
       </c>
       <c r="S16">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="T16">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="U16">
-        <v>500</v>
+        <v>1100</v>
       </c>
       <c r="V16">
-        <v>400</v>
+        <v>800</v>
       </c>
       <c r="W16">
-        <v>1200</v>
+        <v>2600</v>
       </c>
       <c r="X16">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="Y16">
         <v>400</v>
@@ -8482,37 +8556,37 @@
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A17">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17">
         <v>500</v>
       </c>
       <c r="C17">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="D17">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="E17">
+        <v>800</v>
+      </c>
+      <c r="F17">
         <v>500</v>
       </c>
-      <c r="F17">
-        <v>200</v>
-      </c>
       <c r="G17">
-        <v>200</v>
+        <v>900</v>
       </c>
       <c r="H17">
-        <v>500</v>
+        <v>1400</v>
       </c>
       <c r="I17">
-        <v>600</v>
+        <v>2200</v>
       </c>
       <c r="J17">
-        <v>1000</v>
+        <v>1400</v>
       </c>
       <c r="K17">
-        <v>4000</v>
+        <v>4400</v>
       </c>
       <c r="L17">
         <v>1400</v>
@@ -8521,114 +8595,114 @@
         <v>700</v>
       </c>
       <c r="N17">
+        <v>600</v>
+      </c>
+      <c r="O17">
         <v>700</v>
       </c>
-      <c r="O17">
+      <c r="P17">
+        <v>1200</v>
+      </c>
+      <c r="Q17">
+        <v>0</v>
+      </c>
+      <c r="R17">
+        <v>2800</v>
+      </c>
+      <c r="S17">
+        <v>500</v>
+      </c>
+      <c r="T17">
         <v>1300</v>
       </c>
-      <c r="P17">
-        <v>0</v>
-      </c>
-      <c r="Q17">
+      <c r="U17">
+        <v>1600</v>
+      </c>
+      <c r="V17">
+        <v>600</v>
+      </c>
+      <c r="W17">
         <v>1200</v>
       </c>
-      <c r="R17">
-        <v>1500</v>
-      </c>
-      <c r="S17">
-        <v>200</v>
-      </c>
-      <c r="T17">
-        <v>800</v>
-      </c>
-      <c r="U17">
-        <v>1100</v>
-      </c>
-      <c r="V17">
-        <v>800</v>
-      </c>
-      <c r="W17">
-        <v>2600</v>
-      </c>
       <c r="X17">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="Y17">
-        <v>400</v>
+        <v>300</v>
       </c>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A18">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B18">
+        <v>400</v>
+      </c>
+      <c r="C18">
+        <v>200</v>
+      </c>
+      <c r="D18">
+        <v>100</v>
+      </c>
+      <c r="E18">
         <v>500</v>
       </c>
-      <c r="C18">
-        <v>400</v>
-      </c>
-      <c r="D18">
+      <c r="F18">
         <v>200</v>
       </c>
-      <c r="E18">
-        <v>800</v>
-      </c>
-      <c r="F18">
+      <c r="G18">
         <v>500</v>
       </c>
-      <c r="G18">
+      <c r="H18">
+        <v>1000</v>
+      </c>
+      <c r="I18">
+        <v>1400</v>
+      </c>
+      <c r="J18">
         <v>900</v>
       </c>
-      <c r="H18">
-        <v>1400</v>
-      </c>
-      <c r="I18">
-        <v>2200</v>
-      </c>
-      <c r="J18">
-        <v>1400</v>
-      </c>
       <c r="K18">
-        <v>4400</v>
+        <v>3900</v>
       </c>
       <c r="L18">
-        <v>1400</v>
+        <v>1000</v>
       </c>
       <c r="M18">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="N18">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="O18">
         <v>700</v>
       </c>
       <c r="P18">
-        <v>1200</v>
+        <v>1500</v>
       </c>
       <c r="Q18">
-        <v>0</v>
+        <v>2800</v>
       </c>
       <c r="R18">
-        <v>2800</v>
+        <v>0</v>
       </c>
       <c r="S18">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="T18">
-        <v>1300</v>
+        <v>1700</v>
       </c>
       <c r="U18">
-        <v>1600</v>
+        <v>1700</v>
       </c>
       <c r="V18">
         <v>600</v>
       </c>
       <c r="W18">
-        <v>1200</v>
+        <v>1700</v>
       </c>
       <c r="X18">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="Y18">
         <v>300</v>
@@ -8636,161 +8710,161 @@
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A19">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B19">
+        <v>100</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>100</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>100</v>
+      </c>
+      <c r="H19">
+        <v>200</v>
+      </c>
+      <c r="I19">
+        <v>300</v>
+      </c>
+      <c r="J19">
+        <v>200</v>
+      </c>
+      <c r="K19">
+        <v>700</v>
+      </c>
+      <c r="L19">
+        <v>200</v>
+      </c>
+      <c r="M19">
+        <v>200</v>
+      </c>
+      <c r="N19">
+        <v>100</v>
+      </c>
+      <c r="O19">
+        <v>100</v>
+      </c>
+      <c r="P19">
+        <v>200</v>
+      </c>
+      <c r="Q19">
+        <v>500</v>
+      </c>
+      <c r="R19">
+        <v>600</v>
+      </c>
+      <c r="S19">
+        <v>0</v>
+      </c>
+      <c r="T19">
+        <v>300</v>
+      </c>
+      <c r="U19">
         <v>400</v>
       </c>
-      <c r="C19">
-        <v>200</v>
-      </c>
-      <c r="D19">
+      <c r="V19">
         <v>100</v>
       </c>
-      <c r="E19">
-        <v>500</v>
-      </c>
-      <c r="F19">
-        <v>200</v>
-      </c>
-      <c r="G19">
-        <v>500</v>
-      </c>
-      <c r="H19">
-        <v>1000</v>
-      </c>
-      <c r="I19">
-        <v>1400</v>
-      </c>
-      <c r="J19">
-        <v>900</v>
-      </c>
-      <c r="K19">
-        <v>3900</v>
-      </c>
-      <c r="L19">
-        <v>1000</v>
-      </c>
-      <c r="M19">
-        <v>600</v>
-      </c>
-      <c r="N19">
-        <v>500</v>
-      </c>
-      <c r="O19">
-        <v>700</v>
-      </c>
-      <c r="P19">
-        <v>1500</v>
-      </c>
-      <c r="Q19">
-        <v>2800</v>
-      </c>
-      <c r="R19">
-        <v>0</v>
-      </c>
-      <c r="S19">
-        <v>600</v>
-      </c>
-      <c r="T19">
-        <v>1700</v>
-      </c>
-      <c r="U19">
-        <v>1700</v>
-      </c>
-      <c r="V19">
-        <v>600</v>
-      </c>
       <c r="W19">
-        <v>1700</v>
+        <v>300</v>
       </c>
       <c r="X19">
-        <v>600</v>
+        <v>100</v>
       </c>
       <c r="Y19">
-        <v>300</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A20">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B20">
+        <v>300</v>
+      </c>
+      <c r="C20">
         <v>100</v>
       </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
       <c r="D20">
         <v>0</v>
       </c>
       <c r="E20">
+        <v>200</v>
+      </c>
+      <c r="F20">
         <v>100</v>
       </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
       <c r="G20">
+        <v>200</v>
+      </c>
+      <c r="H20">
+        <v>400</v>
+      </c>
+      <c r="I20">
+        <v>700</v>
+      </c>
+      <c r="J20">
+        <v>400</v>
+      </c>
+      <c r="K20">
+        <v>1800</v>
+      </c>
+      <c r="L20">
+        <v>400</v>
+      </c>
+      <c r="M20">
+        <v>300</v>
+      </c>
+      <c r="N20">
+        <v>300</v>
+      </c>
+      <c r="O20">
+        <v>300</v>
+      </c>
+      <c r="P20">
+        <v>800</v>
+      </c>
+      <c r="Q20">
+        <v>1300</v>
+      </c>
+      <c r="R20">
+        <v>1700</v>
+      </c>
+      <c r="S20">
+        <v>300</v>
+      </c>
+      <c r="T20">
+        <v>0</v>
+      </c>
+      <c r="U20">
+        <v>1200</v>
+      </c>
+      <c r="V20">
+        <v>400</v>
+      </c>
+      <c r="W20">
+        <v>1200</v>
+      </c>
+      <c r="X20">
+        <v>300</v>
+      </c>
+      <c r="Y20">
         <v>100</v>
-      </c>
-      <c r="H20">
-        <v>200</v>
-      </c>
-      <c r="I20">
-        <v>300</v>
-      </c>
-      <c r="J20">
-        <v>200</v>
-      </c>
-      <c r="K20">
-        <v>700</v>
-      </c>
-      <c r="L20">
-        <v>200</v>
-      </c>
-      <c r="M20">
-        <v>200</v>
-      </c>
-      <c r="N20">
-        <v>100</v>
-      </c>
-      <c r="O20">
-        <v>100</v>
-      </c>
-      <c r="P20">
-        <v>200</v>
-      </c>
-      <c r="Q20">
-        <v>500</v>
-      </c>
-      <c r="R20">
-        <v>600</v>
-      </c>
-      <c r="S20">
-        <v>0</v>
-      </c>
-      <c r="T20">
-        <v>300</v>
-      </c>
-      <c r="U20">
-        <v>400</v>
-      </c>
-      <c r="V20">
-        <v>100</v>
-      </c>
-      <c r="W20">
-        <v>300</v>
-      </c>
-      <c r="X20">
-        <v>100</v>
-      </c>
-      <c r="Y20">
-        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A21">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B21">
         <v>300</v>
@@ -8802,539 +8876,375 @@
         <v>0</v>
       </c>
       <c r="E21">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="F21">
         <v>100</v>
       </c>
       <c r="G21">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="H21">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="I21">
-        <v>700</v>
+        <v>900</v>
       </c>
       <c r="J21">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="K21">
-        <v>1800</v>
+        <v>2500</v>
       </c>
       <c r="L21">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="M21">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="N21">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="O21">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="P21">
-        <v>800</v>
+        <v>1100</v>
       </c>
       <c r="Q21">
-        <v>1300</v>
+        <v>1600</v>
       </c>
       <c r="R21">
         <v>1700</v>
       </c>
       <c r="S21">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="T21">
-        <v>0</v>
+        <v>1200</v>
       </c>
       <c r="U21">
+        <v>0</v>
+      </c>
+      <c r="V21">
         <v>1200</v>
       </c>
-      <c r="V21">
+      <c r="W21">
+        <v>2400</v>
+      </c>
+      <c r="X21">
+        <v>700</v>
+      </c>
+      <c r="Y21">
         <v>400</v>
-      </c>
-      <c r="W21">
-        <v>1200</v>
-      </c>
-      <c r="X21">
-        <v>300</v>
-      </c>
-      <c r="Y21">
-        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A22">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B22">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="C22">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="D22">
         <v>0</v>
       </c>
       <c r="E22">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="F22">
         <v>100</v>
       </c>
       <c r="G22">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="H22">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="I22">
-        <v>900</v>
+        <v>400</v>
       </c>
       <c r="J22">
         <v>300</v>
       </c>
       <c r="K22">
-        <v>2500</v>
+        <v>1200</v>
       </c>
       <c r="L22">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="M22">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="N22">
         <v>600</v>
       </c>
       <c r="O22">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="P22">
-        <v>1100</v>
+        <v>800</v>
       </c>
       <c r="Q22">
-        <v>1600</v>
+        <v>600</v>
       </c>
       <c r="R22">
-        <v>1700</v>
+        <v>600</v>
       </c>
       <c r="S22">
+        <v>100</v>
+      </c>
+      <c r="T22">
         <v>400</v>
       </c>
-      <c r="T22">
+      <c r="U22">
         <v>1200</v>
       </c>
-      <c r="U22">
-        <v>0</v>
-      </c>
       <c r="V22">
-        <v>1200</v>
+        <v>0</v>
       </c>
       <c r="W22">
-        <v>2400</v>
+        <v>1800</v>
       </c>
       <c r="X22">
         <v>700</v>
       </c>
       <c r="Y22">
-        <v>400</v>
+        <v>500</v>
       </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A23">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B23">
+        <v>400</v>
+      </c>
+      <c r="C23">
         <v>100</v>
       </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
       <c r="D23">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="E23">
+        <v>400</v>
+      </c>
+      <c r="F23">
         <v>200</v>
       </c>
-      <c r="F23">
-        <v>100</v>
-      </c>
       <c r="G23">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="H23">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="I23">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="J23">
+        <v>700</v>
+      </c>
+      <c r="K23">
+        <v>2600</v>
+      </c>
+      <c r="L23">
+        <v>1100</v>
+      </c>
+      <c r="M23">
+        <v>700</v>
+      </c>
+      <c r="N23">
+        <v>1300</v>
+      </c>
+      <c r="O23">
+        <v>1200</v>
+      </c>
+      <c r="P23">
+        <v>2600</v>
+      </c>
+      <c r="Q23">
+        <v>1200</v>
+      </c>
+      <c r="R23">
+        <v>1700</v>
+      </c>
+      <c r="S23">
         <v>300</v>
       </c>
-      <c r="K23">
+      <c r="T23">
         <v>1200</v>
       </c>
-      <c r="L23">
-        <v>400</v>
-      </c>
-      <c r="M23">
-        <v>300</v>
-      </c>
-      <c r="N23">
-        <v>600</v>
-      </c>
-      <c r="O23">
-        <v>400</v>
-      </c>
-      <c r="P23">
-        <v>800</v>
-      </c>
-      <c r="Q23">
-        <v>600</v>
-      </c>
-      <c r="R23">
-        <v>600</v>
-      </c>
-      <c r="S23">
-        <v>100</v>
-      </c>
-      <c r="T23">
-        <v>400</v>
-      </c>
       <c r="U23">
-        <v>1200</v>
+        <v>2400</v>
       </c>
       <c r="V23">
-        <v>0</v>
+        <v>1800</v>
       </c>
       <c r="W23">
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="X23">
-        <v>700</v>
+        <v>2100</v>
       </c>
       <c r="Y23">
-        <v>500</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B24">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="C24">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="D24">
         <v>100</v>
       </c>
       <c r="E24">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="F24">
+        <v>100</v>
+      </c>
+      <c r="G24">
+        <v>100</v>
+      </c>
+      <c r="H24">
         <v>200</v>
       </c>
-      <c r="G24">
-        <v>200</v>
-      </c>
-      <c r="H24">
+      <c r="I24">
+        <v>300</v>
+      </c>
+      <c r="J24">
         <v>500</v>
       </c>
-      <c r="I24">
-        <v>500</v>
-      </c>
-      <c r="J24">
-        <v>700</v>
-      </c>
       <c r="K24">
-        <v>2600</v>
+        <v>1800</v>
       </c>
       <c r="L24">
-        <v>1100</v>
+        <v>1300</v>
       </c>
       <c r="M24">
         <v>700</v>
       </c>
       <c r="N24">
-        <v>1300</v>
+        <v>800</v>
       </c>
       <c r="O24">
-        <v>1200</v>
+        <v>1100</v>
       </c>
       <c r="P24">
-        <v>2600</v>
+        <v>1000</v>
       </c>
       <c r="Q24">
-        <v>1200</v>
+        <v>500</v>
       </c>
       <c r="R24">
-        <v>1700</v>
+        <v>600</v>
       </c>
       <c r="S24">
+        <v>100</v>
+      </c>
+      <c r="T24">
         <v>300</v>
       </c>
-      <c r="T24">
-        <v>1200</v>
-      </c>
       <c r="U24">
-        <v>2400</v>
+        <v>700</v>
       </c>
       <c r="V24">
-        <v>1800</v>
+        <v>700</v>
       </c>
       <c r="W24">
-        <v>0</v>
+        <v>2100</v>
       </c>
       <c r="X24">
-        <v>2100</v>
+        <v>0</v>
       </c>
       <c r="Y24">
-        <v>1100</v>
+        <v>700</v>
       </c>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A25">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B25">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E25">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="F25">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G25">
         <v>100</v>
       </c>
       <c r="H25">
+        <v>100</v>
+      </c>
+      <c r="I25">
         <v>200</v>
       </c>
-      <c r="I25">
+      <c r="J25">
+        <v>200</v>
+      </c>
+      <c r="K25">
+        <v>800</v>
+      </c>
+      <c r="L25">
+        <v>600</v>
+      </c>
+      <c r="M25">
+        <v>500</v>
+      </c>
+      <c r="N25">
+        <v>700</v>
+      </c>
+      <c r="O25">
+        <v>400</v>
+      </c>
+      <c r="P25">
+        <v>400</v>
+      </c>
+      <c r="Q25">
         <v>300</v>
       </c>
-      <c r="J25">
+      <c r="R25">
+        <v>300</v>
+      </c>
+      <c r="S25">
+        <v>0</v>
+      </c>
+      <c r="T25">
+        <v>100</v>
+      </c>
+      <c r="U25">
+        <v>400</v>
+      </c>
+      <c r="V25">
         <v>500</v>
       </c>
-      <c r="K25">
-        <v>1800</v>
-      </c>
-      <c r="L25">
-        <v>1300</v>
-      </c>
-      <c r="M25">
+      <c r="W25">
+        <v>1100</v>
+      </c>
+      <c r="X25">
         <v>700</v>
       </c>
-      <c r="N25">
-        <v>800</v>
-      </c>
-      <c r="O25">
-        <v>1100</v>
-      </c>
-      <c r="P25">
-        <v>1000</v>
-      </c>
-      <c r="Q25">
-        <v>500</v>
-      </c>
-      <c r="R25">
-        <v>600</v>
-      </c>
-      <c r="S25">
-        <v>100</v>
-      </c>
-      <c r="T25">
-        <v>300</v>
-      </c>
-      <c r="U25">
-        <v>700</v>
-      </c>
-      <c r="V25">
-        <v>700</v>
-      </c>
-      <c r="W25">
-        <v>2100</v>
-      </c>
-      <c r="X25">
-        <v>0</v>
-      </c>
       <c r="Y25">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A26">
-        <v>24</v>
-      </c>
-      <c r="B26">
-        <v>100</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-      <c r="D26">
-        <v>0</v>
-      </c>
-      <c r="E26">
-        <v>200</v>
-      </c>
-      <c r="F26">
-        <v>0</v>
-      </c>
-      <c r="G26">
-        <v>100</v>
-      </c>
-      <c r="H26">
-        <v>100</v>
-      </c>
-      <c r="I26">
-        <v>200</v>
-      </c>
-      <c r="J26">
-        <v>200</v>
-      </c>
-      <c r="K26">
-        <v>800</v>
-      </c>
-      <c r="L26">
-        <v>600</v>
-      </c>
-      <c r="M26">
-        <v>500</v>
-      </c>
-      <c r="N26">
-        <v>700</v>
-      </c>
-      <c r="O26">
-        <v>400</v>
-      </c>
-      <c r="P26">
-        <v>400</v>
-      </c>
-      <c r="Q26">
-        <v>300</v>
-      </c>
-      <c r="R26">
-        <v>300</v>
-      </c>
-      <c r="S26">
-        <v>0</v>
-      </c>
-      <c r="T26">
-        <v>100</v>
-      </c>
-      <c r="U26">
-        <v>400</v>
-      </c>
-      <c r="V26">
-        <v>500</v>
-      </c>
-      <c r="W26">
-        <v>1100</v>
-      </c>
-      <c r="X26">
-        <v>700</v>
-      </c>
-      <c r="Y26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" t="s">
-        <v>26</v>
-      </c>
-      <c r="B29">
-        <v>13.51785714</v>
-      </c>
-      <c r="C29">
-        <v>29.610775220000001</v>
-      </c>
-      <c r="D29">
-        <v>10.819500980000001</v>
-      </c>
-      <c r="E29">
-        <v>40.430276200000002</v>
-      </c>
-      <c r="F29">
-        <v>1.2583940220000001</v>
-      </c>
-      <c r="G29">
-        <v>15.44642857</v>
-      </c>
-      <c r="H29">
-        <v>16.34642857</v>
-      </c>
-      <c r="I29">
-        <v>32.227305430000001</v>
-      </c>
-      <c r="J29">
-        <v>6.3627373040000004</v>
-      </c>
-      <c r="K29">
-        <v>38.59004273</v>
-      </c>
-      <c r="L29">
-        <v>1.5682273819999999</v>
-      </c>
-      <c r="M29">
-        <v>9.5357142859999993</v>
-      </c>
-    </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" t="s">
-        <v>27</v>
-      </c>
-      <c r="B30">
-        <v>5.1838598170000001</v>
-      </c>
-      <c r="C30">
-        <v>13.714615070000001</v>
-      </c>
-      <c r="D30">
-        <v>5.47143274</v>
-      </c>
-      <c r="E30">
-        <v>18.866093289999998</v>
-      </c>
-      <c r="F30">
-        <v>0.51428322999999998</v>
-      </c>
-      <c r="G30">
-        <v>4.2934184000000002</v>
-      </c>
-      <c r="H30">
-        <v>6.4287129849999998</v>
-      </c>
-      <c r="I30">
-        <v>16.495763239999999</v>
-      </c>
-      <c r="J30">
-        <v>3.9771048879999999</v>
-      </c>
-      <c r="K30">
-        <v>18.315806330000001</v>
-      </c>
-      <c r="L30">
-        <v>0.66214154700000005</v>
-      </c>
-      <c r="M30">
-        <v>4.5804497030000002</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -9349,7 +9259,7 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B1">
         <v>0</v>
@@ -9426,7 +9336,7 @@
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B2">
         <v>539</v>
@@ -9503,7 +9413,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B3">
         <v>341</v>
@@ -9580,7 +9490,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B4">
         <v>332</v>
@@ -9657,7 +9567,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B5">
         <v>345</v>
@@ -9734,7 +9644,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B6">
         <v>361</v>
@@ -9811,7 +9721,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B7">
         <v>402</v>
@@ -9888,7 +9798,7 @@
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B8">
         <v>548</v>

</xml_diff>